<commit_message>
Update to new certificate artwork (v3)
Rebuild the three templates from "certificate templates(3).pdf":

- Content column shifted +5pt in x and the cert-no/QR block moved
  right; recalibrated all field positions in certgen.js LAYOUT
  (name, course/level/hours, period, certificate number, QR).
- New "levels academy." text watermark (shows through behind the
  values, which sit on top).
- Art template (3) now shows the COURSE only — LEVEL and HOURS were
  removed from the design. New 'courseonly' variant replaces
  'nolevel'; its spreadsheet drops the Level/Hours columns and the
  renderer guards the now-absent hours field.

Also: updated clean-templates.py redaction rects for the new layout,
the template-3 sample spreadsheet, the UI template chip, the e2e
variant label, and the README.
</commit_message>
<xml_diff>
--- a/app/samples/certificate-template-3-sample.xlsx
+++ b/app/samples/certificate-template-3-sample.xlsx
@@ -397,14 +397,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:E3"/>
   <cols>
     <col min="1" max="1" width="24.83203125" customWidth="1"/>
     <col min="2" max="2" width="24.83203125" customWidth="1"/>
     <col min="3" max="3" width="24.83203125" customWidth="1"/>
     <col min="4" max="4" width="24.83203125" customWidth="1"/>
     <col min="5" max="5" width="24.83203125" customWidth="1"/>
-    <col min="6" max="6" width="24.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -418,12 +417,9 @@
         <v>Course</v>
       </c>
       <c r="D1" t="str">
-        <v>Hours</v>
+        <v>Start Date</v>
       </c>
       <c r="E1" t="str">
-        <v>Start Date</v>
-      </c>
-      <c r="F1" t="str">
         <v>End Date</v>
       </c>
     </row>
@@ -438,12 +434,9 @@
         <v>General English</v>
       </c>
       <c r="D2" t="str">
-        <v>48</v>
+        <v>2026-01-16</v>
       </c>
       <c r="E2" t="str">
-        <v>2026-01-16</v>
-      </c>
-      <c r="F2" t="str">
         <v>2026-06-16</v>
       </c>
     </row>
@@ -457,19 +450,16 @@
       <c r="C3" t="str">
         <v>General English</v>
       </c>
-      <c r="D3">
-        <v>36</v>
+      <c r="D3" t="str">
+        <v>2026-02-01</v>
       </c>
       <c r="E3" t="str">
-        <v>2026-02-01</v>
-      </c>
-      <c r="F3" t="str">
         <v>2026-07-01</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>